<commit_message>
Auto update RUP 2026-08-27 10:04:00
</commit_message>
<xml_diff>
--- a/output/rup/2026/Rekap RUP Tahun 2026 (2026-08-27).xlsx
+++ b/output/rup/2026/Rekap RUP Tahun 2026 (2026-08-27).xlsx
@@ -513,7 +513,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia - 104575</t>
+          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia - 5.03.5.04.0.00.01.0000</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
@@ -550,7 +550,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Badan Kesatuan Bangsa dan Politik - 104555</t>
+          <t>Badan Kesatuan Bangsa dan Politik - 8.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
@@ -587,7 +587,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Badan Keuangan dan Aset Daerah - 104517</t>
+          <t>Badan Keuangan dan Aset Daerah - 5.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -624,7 +624,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Badan Penanggulangan Bencana Daerah - 104914</t>
+          <t>Badan Penanggulangan Bencana Daerah - 1.05.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -661,7 +661,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Badan Pendapatan Daerah - 106189</t>
+          <t>Badan Pendapatan Daerah - 5.02.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
@@ -698,7 +698,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah - 103214</t>
+          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah - 5.01.5.05.0.00.01.0000</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -735,7 +735,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Balai Latihan Kerja - 318439</t>
+          <t>Balai Latihan Kerja - 2.07.3.32.0.00.01.0001</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -772,7 +772,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Dermaga Indera Sari - 318442</t>
+          <t>Dermaga Indera Sari - 2.15.0.00.0.00.01.0002</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -809,7 +809,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Dinas Kepemudaan dan Olahraga - 106045</t>
+          <t>Dinas Kepemudaan dan Olahraga - 2.19.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
@@ -846,7 +846,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Dinas Kependudukan dan Pencatatan Sipil - 104574</t>
+          <t>Dinas Kependudukan dan Pencatatan Sipil - 2.12.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -883,7 +883,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Dinas Kesehatan - 105026</t>
+          <t>Dinas Kesehatan - 1.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
@@ -920,7 +920,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian - 103858</t>
+          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian - 2.16.2.20.2.21.01.0000</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
@@ -957,7 +957,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Dinas Lingkungan Hidup - 105718</t>
+          <t>Dinas Lingkungan Hidup - 2.11.3.28.0.00.01.0000</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
@@ -994,7 +994,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Dinas Pariwisata - 103774</t>
+          <t>Dinas Pariwisata - 3.26.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
@@ -1031,7 +1031,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Dinas Pekerjaan Umum dan Penataan Ruang - 97761</t>
+          <t>Dinas Pekerjaan Umum dan Penataan Ruang - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
@@ -1068,7 +1068,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Dinas Pemadam Kebakaran dan Penyelamatan - 182831</t>
+          <t>Dinas Pemadam Kebakaran dan Penyelamatan - 1.05.0.00.0.00.03.0000</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
@@ -1105,7 +1105,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Masyarakat dan Desa - 104564</t>
+          <t>Dinas Pemberdayaan Masyarakat dan Desa - 2.13.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
@@ -1142,7 +1142,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana - 105815</t>
+          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana - 2.08.2.14.0.00.01.0000</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
@@ -1179,7 +1179,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu - 105738</t>
+          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu - 2.18.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
@@ -1216,7 +1216,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan dan Kebudayaan - 318415</t>
+          <t>Dinas Pendidikan dan Kebudayaan - 1.01.2.22.0.00.01.0000</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
@@ -1253,7 +1253,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Dinas Perhubungan - 83087</t>
+          <t>Dinas Perhubungan - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
@@ -1290,7 +1290,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Dinas Perikanan dan Ketahanan Pangan - 107807</t>
+          <t>Dinas Perikanan dan Ketahanan Pangan - 2.09.3.25.0.00.01.0000</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
@@ -1327,7 +1327,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah - 104523</t>
+          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
@@ -1364,7 +1364,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Dinas Perpustakaan dan Kearsipan - 101271</t>
+          <t>Dinas Perpustakaan dan Kearsipan - 2.23.2.24.0.00.01.0000</t>
         </is>
       </c>
       <c r="B25" s="3" t="n">
@@ -1401,7 +1401,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Dinas Pertanian - 182444</t>
+          <t>Dinas Pertanian - 3.27.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
@@ -1438,7 +1438,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan - 104572</t>
+          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan - 1.04.2.10.0.00.01.0000</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
@@ -1475,7 +1475,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Dinas Sosial - 104567</t>
+          <t>Dinas Sosial - 1.06.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
@@ -1512,7 +1512,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Dinas Tenaga Kerja dan Transmigrasi - 105354</t>
+          <t>Dinas Tenaga Kerja dan Transmigrasi - 2.07.3.32.0.00.01.0000</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
@@ -1549,7 +1549,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Inspektorat Daerah - 104557</t>
+          <t>Inspektorat Daerah - 6.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
@@ -1586,7 +1586,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Instalasi Farmasi - 318436</t>
+          <t>Instalasi Farmasi - 1.02.0.00.0.00.01.0022</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
@@ -1623,7 +1623,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Selatan - 104549</t>
+          <t>Kecamatan Arut Selatan - 7.01.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
@@ -1660,7 +1660,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Utara - 108527</t>
+          <t>Kecamatan Arut Utara - 7.01.0.00.0.00.04.0000</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
@@ -1697,7 +1697,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Kecamatan Kotawaringin Lama - 106583</t>
+          <t>Kecamatan Kotawaringin Lama - 7.01.0.00.0.00.03.0000</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
@@ -1734,7 +1734,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Kecamatan Kumai - 105380</t>
+          <t>Kecamatan Kumai - 7.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
@@ -1771,7 +1771,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Banteng - 100808</t>
+          <t>Kecamatan Pangkalan Banteng - 7.01.0.00.0.00.06.0000</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
@@ -1808,7 +1808,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Lada - 105333</t>
+          <t>Kecamatan Pangkalan Lada - 7.01.0.00.0.00.05.0000</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
@@ -1845,7 +1845,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Baru - 318455</t>
+          <t>Kelurahan Baru - 7.01.0.00.0.00.02.0007</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
@@ -1882,7 +1882,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Candi - 318446</t>
+          <t>Kelurahan Candi - 7.01.0.00.0.00.01.0001</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
@@ -1919,7 +1919,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Hilir - 318457</t>
+          <t>Kelurahan Kotawaringin Hilir - 7.01.0.00.0.00.03.0002</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
@@ -1956,7 +1956,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Hulu - 318456</t>
+          <t>Kelurahan Kotawaringin Hulu - 7.01.0.00.0.00.03.0001</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
@@ -1993,7 +1993,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Hilir - 318448</t>
+          <t>Kelurahan Kumai Hilir - 7.01.0.00.0.00.01.0003</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
@@ -2030,7 +2030,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Hulu - 318447</t>
+          <t>Kelurahan Kumai Hulu - 7.01.0.00.0.00.01.0002</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
@@ -2067,7 +2067,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Madurejo - 318451</t>
+          <t>Kelurahan Madurejo - 7.01.0.00.0.00.02.0003</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
@@ -2104,7 +2104,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawai - 318450</t>
+          <t>Kelurahan Mendawai - 7.01.0.00.0.00.02.0002</t>
         </is>
       </c>
       <c r="B45" s="3" t="n">
@@ -2141,7 +2141,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawai Seberang - 318449</t>
+          <t>Kelurahan Mendawai Seberang - 7.01.0.00.0.00.02.0001</t>
         </is>
       </c>
       <c r="B46" s="3" t="n">
@@ -2178,7 +2178,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Pangkut - 318458</t>
+          <t>Kelurahan Pangkut - 7.01.0.00.0.00.04.0001</t>
         </is>
       </c>
       <c r="B47" s="3" t="n">
@@ -2215,7 +2215,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Raja - 318453</t>
+          <t>Kelurahan Raja - 7.01.0.00.0.00.02.0005</t>
         </is>
       </c>
       <c r="B48" s="3" t="n">
@@ -2252,7 +2252,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Raja Seberang - 318454</t>
+          <t>Kelurahan Raja Seberang - 7.01.0.00.0.00.02.0006</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
@@ -2289,7 +2289,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Kelurahan Sidorejo - 318452</t>
+          <t>Kelurahan Sidorejo - 7.01.0.00.0.00.02.0004</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
@@ -2326,7 +2326,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Laboratorium Bahan Konstruksi - 318437</t>
+          <t>Laboratorium Bahan Konstruksi - 1.03.0.00.0.00.01.0001</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
@@ -2363,7 +2363,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Laboratorium Kesehatan Daerah - 318417</t>
+          <t>Laboratorium Kesehatan Daerah - 1.02.0.00.0.00.01.0003</t>
         </is>
       </c>
       <c r="B52" s="3" t="n">
@@ -2400,7 +2400,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Laboratorium Lingkungan - 318440</t>
+          <t>Laboratorium Lingkungan - 2.11.0.00.0.00.01.0001</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
@@ -2437,7 +2437,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Pelabuhan Penyeberangan Kumai - 318441</t>
+          <t>Pelabuhan Penyeberangan Kumai - 2.15.0.00.0.00.01.0001</t>
         </is>
       </c>
       <c r="B54" s="3" t="n">
@@ -2474,7 +2474,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Pengembangan Pakan dan Ternak Unggul - 318445</t>
+          <t>Pengembangan Pakan dan Ternak Unggul - 3.27.0.00.0.00.01.0002</t>
         </is>
       </c>
       <c r="B55" s="3" t="n">
@@ -2511,7 +2511,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Pengujian Kendaraan Bermotor - 318443</t>
+          <t>Pengujian Kendaraan Bermotor - 2.15.0.00.0.00.01.0003</t>
         </is>
       </c>
       <c r="B56" s="3" t="n">
@@ -2548,7 +2548,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Selatan - 318418</t>
+          <t>Puskesmas Arut Selatan - 1.02.0.00.0.00.01.0004</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
@@ -2585,7 +2585,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Utara - 318431</t>
+          <t>Puskesmas Arut Utara - 1.02.0.00.0.00.01.0017</t>
         </is>
       </c>
       <c r="B58" s="3" t="n">
@@ -2622,7 +2622,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Ipuh Bangun Jaya - 318435</t>
+          <t>Puskesmas Ipuh Bangun Jaya - 1.02.0.00.0.00.01.0021</t>
         </is>
       </c>
       <c r="B59" s="3" t="n">
@@ -2659,7 +2659,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Karang Mulya - 318430</t>
+          <t>Puskesmas Karang Mulya - 1.02.0.00.0.00.01.0016</t>
         </is>
       </c>
       <c r="B60" s="3" t="n">
@@ -2696,7 +2696,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Kotawaringin Lama - 318433</t>
+          <t>Puskesmas Kotawaringin Lama - 1.02.0.00.0.00.01.0019</t>
         </is>
       </c>
       <c r="B61" s="3" t="n">
@@ -2733,7 +2733,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Kumai - 318424</t>
+          <t>Puskesmas Kumai - 1.02.0.00.0.00.01.0010</t>
         </is>
       </c>
       <c r="B62" s="3" t="n">
@@ -2770,7 +2770,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Kumpai Batu Atas - 318422</t>
+          <t>Puskesmas Kumpai Batu Atas - 1.02.0.00.0.00.01.0008</t>
         </is>
       </c>
       <c r="B63" s="3" t="n">
@@ -2807,7 +2807,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Madurejo - 318419</t>
+          <t>Puskesmas Madurejo - 1.02.0.00.0.00.01.0005</t>
         </is>
       </c>
       <c r="B64" s="3" t="n">
@@ -2844,7 +2844,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Mendawai - 318420</t>
+          <t>Puskesmas Mendawai - 1.02.0.00.0.00.01.0006</t>
         </is>
       </c>
       <c r="B65" s="3" t="n">
@@ -2881,7 +2881,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Natai Pelingkau - 318421</t>
+          <t>Puskesmas Natai Pelingkau - 1.02.0.00.0.00.01.0007</t>
         </is>
       </c>
       <c r="B66" s="3" t="n">
@@ -2918,7 +2918,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Pandu Sanjaya - 318428</t>
+          <t>Puskesmas Pandu Sanjaya - 1.02.0.00.0.00.01.0014</t>
         </is>
       </c>
       <c r="B67" s="3" t="n">
@@ -2955,7 +2955,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Pangkalan Lada - 318427</t>
+          <t>Puskesmas Pangkalan Lada - 1.02.0.00.0.00.01.0013</t>
         </is>
       </c>
       <c r="B68" s="3" t="n">
@@ -2992,7 +2992,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Riam Durian - 318434</t>
+          <t>Puskesmas Riam Durian - 1.02.0.00.0.00.01.0020</t>
         </is>
       </c>
       <c r="B69" s="3" t="n">
@@ -3029,7 +3029,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Runtu - 318423</t>
+          <t>Puskesmas Runtu - 1.02.0.00.0.00.01.0009</t>
         </is>
       </c>
       <c r="B70" s="3" t="n">
@@ -3066,7 +3066,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Sambi - 318432</t>
+          <t>Puskesmas Sambi - 1.02.0.00.0.00.01.0018</t>
         </is>
       </c>
       <c r="B71" s="3" t="n">
@@ -3103,7 +3103,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Semanggang - 318429</t>
+          <t>Puskesmas Semanggang - 1.02.0.00.0.00.01.0015</t>
         </is>
       </c>
       <c r="B72" s="3" t="n">
@@ -3140,7 +3140,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Sungai Rangit - 318426</t>
+          <t>Puskesmas Sungai Rangit - 1.02.0.00.0.00.01.0012</t>
         </is>
       </c>
       <c r="B73" s="3" t="n">
@@ -3177,7 +3177,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Puskesmas Teluk Bogam - 318425</t>
+          <t>Puskesmas Teluk Bogam - 1.02.0.00.0.00.01.0011</t>
         </is>
       </c>
       <c r="B74" s="3" t="n">
@@ -3214,7 +3214,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Rumah Potong Hewan Ruminansia - 318444</t>
+          <t>Rumah Potong Hewan Ruminansia - 3.27.0.00.0.00.01.0001</t>
         </is>
       </c>
       <c r="B75" s="3" t="n">
@@ -3251,7 +3251,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Rumah Sakit Kutaringin - 318416</t>
+          <t>Rumah Sakit Kutaringin - 1.02.0.00.0.00.01.0002</t>
         </is>
       </c>
       <c r="B76" s="3" t="n">
@@ -3288,7 +3288,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Rumah Sakit Umum Daerah Sultan Imanuddin - 97672</t>
+          <t>Rumah Sakit Umum Daerah Sultan Imanuddin - 1.02.0.00.0.00.01.0001</t>
         </is>
       </c>
       <c r="B77" s="3" t="n">
@@ -3325,7 +3325,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Satuan Polisi Pamong Praja - 104525</t>
+          <t>Satuan Polisi Pamong Praja - 1.05.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B78" s="3" t="n">
@@ -3362,7 +3362,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Sekretariat DPRD - 101281</t>
+          <t>Sekretariat DPRD - 4.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B79" s="3" t="n">
@@ -3399,7 +3399,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Sekretariat Daerah - 98763</t>
+          <t>Sekretariat Daerah - 4.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="B80" s="3" t="n">
@@ -3436,7 +3436,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Workshop dan Peralatan Konstruksi - 318438</t>
+          <t>Workshop dan Peralatan Konstruksi - 1.03.0.00.0.00.01.0002</t>
         </is>
       </c>
       <c r="B81" s="3" t="n">

</xml_diff>